<commit_message>
new sim on base case
</commit_message>
<xml_diff>
--- a/case_studies/base_case_00_5_dd/2030/technologies.xlsx
+++ b/case_studies/base_case_00_5_dd/2030/technologies.xlsx
@@ -691,10 +691,10 @@
         <v>0</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>54.48</v>
+        <v>51.54</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>153.14</v>
+        <v>140.61</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>0</v>
@@ -712,13 +712,13 @@
         <v>0</v>
       </c>
       <c r="P2" s="3" t="n">
-        <v>137.9</v>
+        <v>130.46</v>
       </c>
       <c r="Q2" s="3" t="n">
         <v>184.21</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>37.46</v>
+        <v>35.44</v>
       </c>
       <c r="S2" s="3" t="n">
         <v>21.27</v>
@@ -730,10 +730,10 @@
         <v>0</v>
       </c>
       <c r="V2" s="3" t="n">
-        <v>46.73</v>
+        <v>69.83</v>
       </c>
       <c r="W2" s="3" t="n">
-        <v>24.75</v>
+        <v>16.44</v>
       </c>
       <c r="X2" s="3" t="n">
         <v>0</v>
@@ -1079,10 +1079,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>67.88</v>
+        <v>67.83</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>117.49</v>
+        <v>117.43</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>42.99</v>
@@ -1100,16 +1100,16 @@
         <v>0</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>121.74</v>
+        <v>121.61</v>
       </c>
       <c r="Q6" s="3" t="n">
-        <v>135.21</v>
+        <v>135.45</v>
       </c>
       <c r="R6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>9.16</v>
+        <v>9.42</v>
       </c>
       <c r="T6" s="3" t="n">
         <v>95.54000000000001</v>
@@ -1203,10 +1203,10 @@
         <v>0</v>
       </c>
       <c r="R7" s="5" t="n">
-        <v>19.77</v>
+        <v>19.87</v>
       </c>
       <c r="S7" s="5" t="n">
-        <v>15.76</v>
+        <v>15.58</v>
       </c>
       <c r="T7" s="5" t="n">
         <v>48.52</v>
@@ -1215,10 +1215,10 @@
         <v>0</v>
       </c>
       <c r="V7" s="5" t="n">
-        <v>1.14</v>
+        <v>1.73</v>
       </c>
       <c r="W7" s="5" t="n">
-        <v>19.46</v>
+        <v>19.4</v>
       </c>
       <c r="X7" s="5" t="n">
         <v>0</v>

</xml_diff>